<commit_message>
fix test agent 3
</commit_message>
<xml_diff>
--- a/agent3_ground_truth_template.xlsx
+++ b/agent3_ground_truth_template.xlsx
@@ -817,7 +817,7 @@
     <col width="30" customWidth="1" min="13" max="13"/>
     <col width="17" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="17" customWidth="1" min="16" max="16"/>
     <col width="29" customWidth="1" min="17" max="17"/>
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="27" customWidth="1" min="19" max="19"/>
@@ -5214,7 +5214,7 @@
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
         <is>
-          <t>Cambridge CAE: N/A</t>
+          <t>Level: C1</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
@@ -5318,7 +5318,7 @@
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
         <is>
-          <t>Cambridge CAE: N/A</t>
+          <t>Level: C1</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
@@ -5422,7 +5422,7 @@
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr">
         <is>
-          <t>Cambridge CAE: N/A</t>
+          <t>Level: C1</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
@@ -5526,7 +5526,7 @@
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr">
         <is>
-          <t>Cambridge CAE: N/A</t>
+          <t>Level: C1</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
@@ -5630,7 +5630,7 @@
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr">
         <is>
-          <t>Cambridge CAE: N/A</t>
+          <t>Level: C1</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
@@ -5734,7 +5734,7 @@
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr">
         <is>
-          <t>Cambridge CAE: N/A</t>
+          <t>Level: C1</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
@@ -5838,7 +5838,7 @@
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr">
         <is>
-          <t>Cambridge CAE: N/A</t>
+          <t>Level: C1</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
@@ -5942,7 +5942,7 @@
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr">
         <is>
-          <t>Cambridge CAE: N/A</t>
+          <t>Level: C1</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
@@ -6046,7 +6046,7 @@
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr">
         <is>
-          <t>Cambridge CAE: N/A</t>
+          <t>Level: C1</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
@@ -6150,7 +6150,7 @@
       <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr">
         <is>
-          <t>Cambridge CAE: N/A</t>
+          <t>Level: C1</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
@@ -6254,7 +6254,7 @@
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr">
         <is>
-          <t>Cambridge CAE: N/A</t>
+          <t>Level: C1</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
@@ -6358,7 +6358,7 @@
       <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr">
         <is>
-          <t>Cambridge CAE: N/A</t>
+          <t>Level: C1</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
@@ -6462,7 +6462,7 @@
       <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr">
         <is>
-          <t>Cambridge CAE: N/A</t>
+          <t>Level: C1</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
@@ -6566,7 +6566,7 @@
       <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr">
         <is>
-          <t>Cambridge CAE: N/A</t>
+          <t>Level: C1</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
@@ -6670,7 +6670,7 @@
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr">
         <is>
-          <t>Cambridge CAE: N/A</t>
+          <t>Level: C1</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
@@ -6774,7 +6774,7 @@
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr">
         <is>
-          <t>Cambridge CAE: N/A</t>
+          <t>Level: C1</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
@@ -6878,7 +6878,7 @@
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr">
         <is>
-          <t>Cambridge CAE: N/A</t>
+          <t>Level: C1</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
@@ -6982,7 +6982,7 @@
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr">
         <is>
-          <t>Cambridge CAE: N/A</t>
+          <t>Level: C1</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
@@ -7086,7 +7086,7 @@
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr">
         <is>
-          <t>Cambridge CAE: N/A</t>
+          <t>Level: C1</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
@@ -7190,7 +7190,7 @@
       <c r="O61" t="inlineStr"/>
       <c r="P61" t="inlineStr">
         <is>
-          <t>Cambridge CAE: N/A</t>
+          <t>Level: C1</t>
         </is>
       </c>
       <c r="Q61" t="inlineStr">

</xml_diff>